<commit_message>
REG1 value changed from 0.20 to 0.50
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_CO2_TAX.xlsx
+++ b/SuppXLS/Scen_CO2_TAX.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22730"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Training material\DemoS_012\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{086E86E5-D905-4F4C-9C4C-6B4CF20FF611}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1905" yWindow="1905" windowWidth="21600" windowHeight="11385"/>
+    <workbookView xWindow="1905" yWindow="1905" windowWidth="21600" windowHeight="11385" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="CO2_Tax" sheetId="2" r:id="rId1"/>
+    <sheet name="CO2_Tax" sheetId="2" r:id="rId3"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -28,18 +28,17 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Maurizio Gargiulo</author>
   </authors>
   <commentList>
-    <comment ref="B2" authorId="0" shapeId="0">
+    <comment ref="B2" authorId="0">
       <text>
         <r>
           <rPr>
             <b/>
             <sz val="8"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -54,56 +53,62 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
   <si>
+    <t>REG2</t>
+  </si>
+  <si>
+    <t>Attribute</t>
+  </si>
+  <si>
+    <t>Cset_CN</t>
+  </si>
+  <si>
+    <t>\I:Unit</t>
+  </si>
+  <si>
+    <t>COM_TAXNET</t>
+  </si>
+  <si>
+    <t>Meuro/kt</t>
+  </si>
+  <si>
+    <t>TOTCO2</t>
+  </si>
+  <si>
     <t>Year</t>
   </si>
   <si>
-    <t>Cset_CN</t>
-  </si>
-  <si>
-    <t>Attribute</t>
+    <t>REG1</t>
+  </si>
+  <si>
+    <t>~TFM_INS</t>
+  </si>
+  <si>
+    <t>Trans - Insert</t>
+  </si>
+  <si>
+    <t>TimeSlice</t>
   </si>
   <si>
     <t>LimType</t>
-  </si>
-  <si>
-    <t>~TFM_INS</t>
-  </si>
-  <si>
-    <t>TimeSlice</t>
-  </si>
-  <si>
-    <t>Trans - Insert</t>
-  </si>
-  <si>
-    <t>REG2</t>
-  </si>
-  <si>
-    <t>REG1</t>
-  </si>
-  <si>
-    <t>COM_TAXNET</t>
-  </si>
-  <si>
-    <t>TOTCO2</t>
-  </si>
-  <si>
-    <t>Meuro/kt</t>
-  </si>
-  <si>
-    <t>\I:Unit</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -132,7 +137,6 @@
     <font>
       <b/>
       <sz val="8"/>
-      <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
@@ -158,7 +162,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
+        <fgColor theme="6" tint="0.799979984760284"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -175,50 +179,148 @@
       <left/>
       <right/>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="medium">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
       <top style="medium">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+  <cellStyleXfs count="22">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="8">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10" xfId="1"/>
-    <cellStyle name="Normale_Scen_UC_IND-StrucConst" xfId="2"/>
+    <cellStyle name="Percent" xfId="15" builtinId="5"/>
+    <cellStyle name="Currency" xfId="16" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="17" builtinId="7"/>
+    <cellStyle name="Comma" xfId="18" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="19" builtinId="6"/>
+    <cellStyle name="Normal 10" xfId="20"/>
+    <cellStyle name="Normale_Scen_UC_IND-StrucConst" xfId="21"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -231,7 +333,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -245,12 +347,12 @@
       <xdr:row>11</xdr:row>
       <xdr:rowOff>111125</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="">
+    <xdr:sp>
       <xdr:nvSpPr>
         <xdr:cNvPr id="2" name="TextBox 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1D26FDE8-053E-46B0-9D54-97A4B095E765}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1d26fde8-053e-46b0-9d54-97a4b095e765}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -258,12 +360,10 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="611188" y="1341438"/>
-          <a:ext cx="4754562" cy="492125"/>
+          <a:off x="609600" y="1724025"/>
+          <a:ext cx="4752975" cy="495300"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
+        <a:prstGeom prst="rect"/>
         <a:solidFill>
           <a:schemeClr val="accent6">
             <a:lumMod val="20000"/>
@@ -272,7 +372,7 @@
         </a:solidFill>
         <a:ln w="9525" cmpd="sng">
           <a:solidFill>
-            <a:schemeClr val="lt1">
+            <a:schemeClr val="bg1">
               <a:shade val="50000"/>
             </a:schemeClr>
           </a:solidFill>
@@ -280,26 +380,27 @@
       </xdr:spPr>
       <xdr:style>
         <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:lnRef>
         <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:fillRef>
         <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:effectRef>
         <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
+          <a:schemeClr val="tx1"/>
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
         <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
         <a:lstStyle/>
         <a:p>
+          <a:pPr/>
           <a:r>
             <a:rPr lang="en-GB" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -311,7 +412,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -323,7 +424,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -335,7 +436,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -347,7 +448,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -357,6 +458,9 @@
             <a:t>.</a:t>
           </a:r>
           <a:endParaRPr lang="en-GB">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
             <a:effectLst/>
           </a:endParaRPr>
         </a:p>
@@ -687,104 +791,104 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="10.7109375" customWidth="1"/>
-    <col min="8" max="8" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.1428571428571" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85714285714286" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.2857142857143" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.14285714285714" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="10.7142857142857" customWidth="1"/>
+    <col min="8" max="8" width="8.42857142857143" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="15">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:8" ht="15">
       <c r="B2" s="1" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:8" ht="15.75" thickBot="1">
       <c r="B3" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>8</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:8" ht="15">
       <c r="B4" s="6" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="C4" s="6"/>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
       <c r="F4" s="6" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="H4" s="7"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="4:8" ht="15">
       <c r="D5" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E5">
         <v>2015</v>
       </c>
       <c r="F5" s="8">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="G5" s="8">
-        <v>1.4999999999999999E-2</v>
+        <v>0.015</v>
       </c>
       <c r="H5" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="4:8" ht="15">
       <c r="D6" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E6">
         <v>2050</v>
       </c>
       <c r="F6" s="8">
-        <v>0.1</v>
+        <v>0.10</v>
       </c>
       <c r="G6" s="8">
-        <v>0.1</v>
+        <v>0.10</v>
       </c>
       <c r="H6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="4:8" ht="15">
       <c r="D7" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -796,12 +900,12 @@
         <v>5</v>
       </c>
       <c r="H7" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>